<commit_message>
WIP: statement-facsimile engine plan + Excel source-of-truth files
Checkpoint on a WIP branch — NOT to be folded into Rick until the facsimile rebuild is complete. Contains the Act-1 A-E fold-in (M3/M4 pages, engine, shared.*, design docs; 43-2 deleted; Bike-Repair.xlsx replaced by Bike-Repair-End.xlsx), Rick's four source-of-truth .xlsx, and the numbered Statement-Facsimile-Engine-Plan.md.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Cash-Flow-Steps.xlsx
+++ b/Cash-Flow-Steps.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ra1/Courses-Local/Instructional_Redesign_v2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_E7934C45DC22546CAA08204013B676CCFDD802A9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23DCD215-2F3C-9245-BD55-B6986F27E67F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="44480" yWindow="4320" windowWidth="24600" windowHeight="20940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11680" yWindow="3800" windowWidth="24600" windowHeight="20940" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="0 · Data copied in" sheetId="1" r:id="rId1"/>
@@ -204,8 +204,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="3">
+    <numFmt numFmtId="41" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="\$#,##0;\(\$#,##0\)"/>
+    <numFmt numFmtId="168" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -254,7 +256,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -317,7 +319,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -335,7 +337,10 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="168" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1585,7 +1590,7 @@
       <c r="B5" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="13">
         <v>5500</v>
       </c>
     </row>
@@ -1593,7 +1598,7 @@
       <c r="B6" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="15">
         <v>-1200</v>
       </c>
     </row>
@@ -1601,7 +1606,7 @@
       <c r="B7" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="15">
         <v>-1950</v>
       </c>
     </row>
@@ -1610,7 +1615,7 @@
         <v>40</v>
       </c>
       <c r="C8" s="11"/>
-      <c r="D8" s="12">
+      <c r="D8" s="14">
         <f>SUM(D5:D7)</f>
         <v>2350</v>
       </c>
@@ -1626,7 +1631,7 @@
       <c r="B11" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D11" s="13">
         <v>-400</v>
       </c>
     </row>
@@ -1635,7 +1640,7 @@
         <v>42</v>
       </c>
       <c r="C12" s="11"/>
-      <c r="D12" s="12">
+      <c r="D12" s="14">
         <f>SUM(D11:D11)</f>
         <v>-400</v>
       </c>
@@ -1651,7 +1656,7 @@
       <c r="B15" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="D15" s="4">
+      <c r="D15" s="13">
         <v>-2030</v>
       </c>
     </row>
@@ -1659,7 +1664,7 @@
       <c r="B16" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="D16" s="4">
+      <c r="D16" s="15">
         <v>-600</v>
       </c>
     </row>
@@ -1668,7 +1673,7 @@
         <v>44</v>
       </c>
       <c r="C17" s="11"/>
-      <c r="D17" s="12">
+      <c r="D17" s="14">
         <f>SUM(D15:D16)</f>
         <v>-2630</v>
       </c>
@@ -1678,7 +1683,7 @@
         <v>45</v>
       </c>
       <c r="C19" s="11"/>
-      <c r="D19" s="12">
+      <c r="D19" s="14">
         <f>D8+D12+D17</f>
         <v>-680</v>
       </c>
@@ -1687,7 +1692,7 @@
       <c r="B20" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D20" s="13">
+      <c r="D20" s="16">
         <v>1300</v>
       </c>
     </row>
@@ -1696,7 +1701,7 @@
         <v>53</v>
       </c>
       <c r="C21" s="11"/>
-      <c r="D21" s="12">
+      <c r="D21" s="14">
         <f>D20+D19</f>
         <v>620</v>
       </c>

</xml_diff>